<commit_message>
Add repository-specific replication discovery
</commit_message>
<xml_diff>
--- a/outputs/research_data_enrichment/Forschungsdaten_2024-heute_3_Sheets_konsolidiert_geprueft.xlsx
+++ b/outputs/research_data_enrichment/Forschungsdaten_2024-heute_3_Sheets_konsolidiert_geprueft.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R597e2ffc7c454a30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsdaten" sheetId="2" r:id="R4b6eba3876b74760"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsgruppen" sheetId="3" r:id="R136cd4ea0bd14fac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R17c0037bd173470d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsdaten" sheetId="2" r:id="Re344329f36494409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsgruppen" sheetId="3" r:id="R51d1768a4f474d65"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -606,7 +606,7 @@
         <x:v>Forschungsdaten: ja</x:v>
       </x:c>
       <x:c r="B5" s="14" t="n">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -614,7 +614,7 @@
         <x:v>Forschungsdaten: nein</x:v>
       </x:c>
       <x:c r="B6" s="14" t="n">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -622,7 +622,7 @@
         <x:v>Abdeckungsquote</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:v>0.17562724014336917</x:v>
+        <x:v>0.1827956989247312</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -630,7 +630,7 @@
         <x:v>Verifizierte Forschungsdatenlinks</x:v>
       </x:c>
       <x:c r="B8" s="14" t="n">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -702,7 +702,7 @@
         <x:v>Quellenpriorität</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
-        <x:v>1. PuRe; 2. explizite Data-Availability-Aussagen; 3. DataCite/OSF/B2FIND mit engem Titel- oder Autor:innenbezug</x:v>
+        <x:v>1. gepflegte PuRe-Links; 2. explizite Data-Availability-Aussagen; 3. Repositorien mit engem Titel-/Autor:innenbezug und geprüften Datendateien</x:v>
       </x:c>
       <x:c r="C17" s="23" t="str"/>
       <x:c r="D17" s="23" t="str"/>
@@ -723,10 +723,10 @@
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="22" t="str">
-        <x:v>OSF-Prüfung</x:v>
+        <x:v>Dateiprüfung</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
-        <x:v>Dateistruktur rekursiv über OSF-API; mindestens eine erkennbare Datendatei oder ein expliziter Data-Availability-Nachweis</x:v>
+        <x:v>OSF- und GitHub-Dateibäume rekursiv über die jeweilige API; Zenodo-Archive werden bis auf Dateiebene geprüft</x:v>
       </x:c>
       <x:c r="C19" s="23" t="str"/>
       <x:c r="D19" s="23" t="str"/>
@@ -4019,7 +4019,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ33" s="31" t="str">
-        <x:v>GitHub-README mit exaktem Publikationstitel und geprüften Datendateien</x:v>
+        <x:v>GitHub-README mit exaktem Publikationstitel und geprüften Datendateien; 55 Datendatei(en) über GitHub-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
@@ -13466,7 +13466,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ142" s="31" t="str">
-        <x:v>GitHub-README mit exaktem Publikationstitel und geprüften Datendateien</x:v>
+        <x:v>GitHub-README mit exaktem Publikationstitel und geprüften Datendateien; 7424 Datendatei(en) über GitHub-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="34" customHeight="1">
@@ -14948,19 +14948,27 @@
       <x:c r="J160" s="31" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="K160" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K160" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L160" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M160" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N160" s="37" t="str"/>
-      <x:c r="O160" s="31" t="str"/>
-      <x:c r="P160" s="31" t="str"/>
-      <x:c r="Q160" s="31" t="str"/>
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="N160" s="37" t="str">
+        <x:v>https://github.com/nbreznau/how_many_replicators</x:v>
+      </x:c>
+      <x:c r="O160" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P160" s="31" t="str">
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="Q160" s="31" t="str">
+        <x:v>HTTP 200; HTTP</x:v>
+      </x:c>
       <x:c r="R160" s="37" t="str"/>
       <x:c r="S160" s="31" t="str"/>
       <x:c r="T160" s="31" t="str"/>
@@ -14997,10 +15005,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY160" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ160" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Link aus expliziter Data-Availability-Statement; 202 Datendatei(en) über GitHub-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="34" customHeight="1">
@@ -23402,19 +23410,27 @@
       <x:c r="J258" s="31" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="K258" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K258" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L258" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M258" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N258" s="37" t="str"/>
-      <x:c r="O258" s="31" t="str"/>
-      <x:c r="P258" s="31" t="str"/>
-      <x:c r="Q258" s="31" t="str"/>
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="N258" s="37" t="str">
+        <x:v>https://zenodo.org/records/10438859</x:v>
+      </x:c>
+      <x:c r="O258" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P258" s="31" t="str">
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="Q258" s="31" t="str">
+        <x:v>HTTP 200; HTTP</x:v>
+      </x:c>
       <x:c r="R258" s="37" t="str"/>
       <x:c r="S258" s="31" t="str"/>
       <x:c r="T258" s="31" t="str"/>
@@ -23451,10 +23467,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY258" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ258" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Zenodo-Replikationspaket mit Titel-/Autor:innen-Match und geprüften Datendateien</x:v>
       </x:c>
     </x:row>
     <x:row r="259" ht="34" customHeight="1">
@@ -25344,7 +25360,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b9cfc2a5bd847f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a17a9d77f2d4de0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25427,19 +25443,19 @@
         <x:v>118</x:v>
       </x:c>
       <x:c r="C5" s="31" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="31" t="n">
-        <x:v>100</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="E5" s="49" t="n">
-        <x:v>0.15254237288135594</x:v>
+        <x:v>0.16101694915254236</x:v>
       </x:c>
       <x:c r="F5" s="31" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="G5" s="31" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
@@ -25611,13 +25627,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="34" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D13" s="34" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D13" s="34" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="E13" s="50" t="n">
-        <x:v>0.3333333333333333</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="F13" s="34" t="n">
         <x:v>0</x:v>
@@ -25659,7 +25675,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4c3ee62b1474b71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff384e42b90b4a7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update consolidated research data report
</commit_message>
<xml_diff>
--- a/outputs/research_data_enrichment/Forschungsdaten_2024-heute_3_Sheets_konsolidiert_geprueft.xlsx
+++ b/outputs/research_data_enrichment/Forschungsdaten_2024-heute_3_Sheets_konsolidiert_geprueft.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R17c0037bd173470d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsdaten" sheetId="2" r:id="Re344329f36494409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsgruppen" sheetId="3" r:id="R51d1768a4f474d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R1290edaebf634759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsdaten" sheetId="2" r:id="Rd7a69ad6e70d4438"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forschungsgruppen" sheetId="3" r:id="R990fdc6efef6495c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -606,7 +606,7 @@
         <x:v>Forschungsdaten: ja</x:v>
       </x:c>
       <x:c r="B5" s="14" t="n">
-        <x:v>51</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -614,7 +614,7 @@
         <x:v>Forschungsdaten: nein</x:v>
       </x:c>
       <x:c r="B6" s="14" t="n">
-        <x:v>228</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -622,7 +622,7 @@
         <x:v>Abdeckungsquote</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:v>0.1827956989247312</x:v>
+        <x:v>0.21505376344086022</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -630,7 +630,7 @@
         <x:v>Verifizierte Forschungsdatenlinks</x:v>
       </x:c>
       <x:c r="B8" s="14" t="n">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -750,7 +750,7 @@
         <x:v>Zugang</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
-        <x:v>Paywall, Login, Embargo und Zugriffsbeschränkung erscheinen je Link in einer eigenen Spalte</x:v>
+        <x:v>Paywall, Login, Embargo, Zustimmungspflichten und View-only-Zugänge erscheinen je Link in einer eigenen Spalte</x:v>
       </x:c>
       <x:c r="C21" s="23" t="str"/>
       <x:c r="D21" s="23" t="str"/>
@@ -786,7 +786,7 @@
         <x:v>Gelb</x:v>
       </x:c>
       <x:c r="B26" s="14" t="str">
-        <x:v>Paywall, Login, Embargo oder Zugriffsbeschränkung</x:v>
+        <x:v>Paywall, Login, Embargo, Zustimmungspflicht oder View-only-Zugang</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1587,27 +1587,35 @@
         <x:v>ja</x:v>
       </x:c>
       <x:c r="L7" s="41" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M7" s="31" t="str">
-        <x:v>offen</x:v>
+        <x:v>Paywall/Login oder Zugriffsschutz; offen</x:v>
       </x:c>
       <x:c r="N7" s="37" t="str">
-        <x:v>https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/DCSR0N</x:v>
+        <x:v>https://dataverse.harvard.edu/citation?persistentId=doi:10.7910/DVN/DCSR0N</x:v>
       </x:c>
       <x:c r="O7" s="31" t="str">
         <x:v>PuRe</x:v>
       </x:c>
-      <x:c r="P7" s="31" t="str">
+      <x:c r="P7" s="39" t="str">
+        <x:v>Paywall/Login oder Zugriffsschutz</x:v>
+      </x:c>
+      <x:c r="Q7" s="31" t="str">
+        <x:v>HTTP 403; Playwright</x:v>
+      </x:c>
+      <x:c r="R7" s="37" t="str">
+        <x:v>https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/DCSR0N</x:v>
+      </x:c>
+      <x:c r="S7" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="T7" s="31" t="str">
         <x:v>offen</x:v>
       </x:c>
-      <x:c r="Q7" s="31" t="str">
+      <x:c r="U7" s="31" t="str">
         <x:v>HTTP 202; Playwright</x:v>
       </x:c>
-      <x:c r="R7" s="37" t="str"/>
-      <x:c r="S7" s="31" t="str"/>
-      <x:c r="T7" s="31" t="str"/>
-      <x:c r="U7" s="31" t="str"/>
       <x:c r="V7" s="37" t="str"/>
       <x:c r="W7" s="31" t="str"/>
       <x:c r="X7" s="31" t="str"/>
@@ -1643,7 +1651,7 @@
         <x:v>Playwright</x:v>
       </x:c>
       <x:c r="AZ7" s="31" t="str">
-        <x:v>Kuratiertes PuRe-Forschungsdatenfeld</x:v>
+        <x:v>Kuratiertes PuRe-Forschungsdatenfeld; Landingpage antwortet mit HTTP 403 und ist zugriffsgeschützt; Titel-/Autor:innen-Match (1.00)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -2186,7 +2194,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="M13" s="31" t="str">
-        <x:v>offen</x:v>
+        <x:v>offen über View-only-Link</x:v>
       </x:c>
       <x:c r="N13" s="37" t="str">
         <x:v>https://osf.io/b8zp4/?view_only=f331e7a632e54a6fbaf5763175393150</x:v>
@@ -2194,8 +2202,8 @@
       <x:c r="O13" s="31" t="str">
         <x:v>PuRe</x:v>
       </x:c>
-      <x:c r="P13" s="31" t="str">
-        <x:v>offen</x:v>
+      <x:c r="P13" s="39" t="str">
+        <x:v>offen über View-only-Link</x:v>
       </x:c>
       <x:c r="Q13" s="31" t="str">
         <x:v>HTTP 200; HTTP</x:v>
@@ -2280,7 +2288,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="M14" s="31" t="str">
-        <x:v>offen</x:v>
+        <x:v>offen über View-only-Link; offen</x:v>
       </x:c>
       <x:c r="N14" s="37" t="str">
         <x:v>https://osf.io/4n8hy/?view_only=fb104cd14ba548e0b01b997908fdbeb8</x:v>
@@ -2288,8 +2296,8 @@
       <x:c r="O14" s="31" t="str">
         <x:v>PuRe</x:v>
       </x:c>
-      <x:c r="P14" s="31" t="str">
-        <x:v>offen</x:v>
+      <x:c r="P14" s="39" t="str">
+        <x:v>offen über View-only-Link</x:v>
       </x:c>
       <x:c r="Q14" s="31" t="str">
         <x:v>HTTP 200; HTTP</x:v>
@@ -2341,7 +2349,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ14" s="31" t="str">
-        <x:v>Kuratiertes PuRe-Forschungsdatenfeld; Link aus Data-Availability-Abschnitt des öffentlichen PuRe-Volltexts</x:v>
+        <x:v>Kuratiertes PuRe-Forschungsdatenfeld; Link aus Data-Availability-Abschnitt des öffentlichen PuRe-Volltexts; 1 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -2883,7 +2891,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ20" s="31" t="str">
-        <x:v>Titel-/Autor:innen-Match (1.00)</x:v>
+        <x:v>Titel-/Autor:innen-Match (1.00); 1 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
@@ -3493,7 +3501,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ27" s="31" t="str">
-        <x:v>Titel-/Autor:innen-Match (1.00)</x:v>
+        <x:v>Titel-/Autor:innen-Match (1.00); 208 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="34" customHeight="1">
@@ -3587,7 +3595,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ28" s="31" t="str">
-        <x:v>Titel-/Autor:innen-Match (1.00)</x:v>
+        <x:v>Titel-/Autor:innen-Match (1.00); 7 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
@@ -3791,19 +3799,27 @@
       <x:c r="J31" s="31" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="K31" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K31" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L31" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M31" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N31" s="37" t="str"/>
-      <x:c r="O31" s="31" t="str"/>
-      <x:c r="P31" s="31" t="str"/>
-      <x:c r="Q31" s="31" t="str"/>
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="N31" s="37" t="str">
+        <x:v>https://services.informs.org/dataset/mnsc/download.php?doi=mnsc.2022.00990</x:v>
+      </x:c>
+      <x:c r="O31" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P31" s="39" t="str">
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="Q31" s="31" t="str">
+        <x:v>HTTP 200; Playwright</x:v>
+      </x:c>
       <x:c r="R31" s="37" t="str"/>
       <x:c r="S31" s="31" t="str"/>
       <x:c r="T31" s="31" t="str"/>
@@ -3840,10 +3856,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY31" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>Playwright</x:v>
       </x:c>
       <x:c r="AZ31" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Offizielles INFORMS-Replikationsarchiv mit geprüften Datendateien</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
@@ -3877,19 +3893,27 @@
       <x:c r="J32" s="31" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="K32" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K32" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L32" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M32" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N32" s="37" t="str"/>
-      <x:c r="O32" s="31" t="str"/>
-      <x:c r="P32" s="31" t="str"/>
-      <x:c r="Q32" s="31" t="str"/>
+        <x:v>offen über View-only-Link</x:v>
+      </x:c>
+      <x:c r="N32" s="37" t="str">
+        <x:v>https://osf.io/yef3k/?view_only=6d8e23c8ced94e3680c5f459a471fd1f</x:v>
+      </x:c>
+      <x:c r="O32" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P32" s="39" t="str">
+        <x:v>offen über View-only-Link</x:v>
+      </x:c>
+      <x:c r="Q32" s="31" t="str">
+        <x:v>HTTP 200; HTTP</x:v>
+      </x:c>
       <x:c r="R32" s="37" t="str"/>
       <x:c r="S32" s="31" t="str"/>
       <x:c r="T32" s="31" t="str"/>
@@ -3926,10 +3950,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY32" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ32" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Wiley-Datenverfügbarkeitsaussage mit rekursiv geprüften OSF-Datendateien; 17 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
@@ -5185,10 +5209,10 @@
         <x:v>ja</x:v>
       </x:c>
       <x:c r="L47" s="41" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M47" s="31" t="str">
-        <x:v>offen</x:v>
+        <x:v>offen über View-only-Link</x:v>
       </x:c>
       <x:c r="N47" s="37" t="str">
         <x:v>https://osf.io/s43na/?view_only=ecc07a520bf64f9397adb25d70c7deb5</x:v>
@@ -5196,24 +5220,16 @@
       <x:c r="O47" s="31" t="str">
         <x:v>Provider</x:v>
       </x:c>
-      <x:c r="P47" s="31" t="str">
-        <x:v>offen</x:v>
+      <x:c r="P47" s="39" t="str">
+        <x:v>offen über View-only-Link</x:v>
       </x:c>
       <x:c r="Q47" s="31" t="str">
         <x:v>HTTP 200; HTTP</x:v>
       </x:c>
-      <x:c r="R47" s="37" t="str">
-        <x:v>https://osf.io/d2fex/?view_only=daca41c653574a8aa1fb40d6b6a7f46c</x:v>
-      </x:c>
-      <x:c r="S47" s="31" t="str">
-        <x:v>Provider</x:v>
-      </x:c>
-      <x:c r="T47" s="31" t="str">
-        <x:v>offen</x:v>
-      </x:c>
-      <x:c r="U47" s="31" t="str">
-        <x:v>HTTP 200; HTTP</x:v>
-      </x:c>
+      <x:c r="R47" s="37" t="str"/>
+      <x:c r="S47" s="31" t="str"/>
+      <x:c r="T47" s="31" t="str"/>
+      <x:c r="U47" s="31" t="str"/>
       <x:c r="V47" s="37" t="str"/>
       <x:c r="W47" s="31" t="str"/>
       <x:c r="X47" s="31" t="str"/>
@@ -5249,7 +5265,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ47" s="31" t="str">
-        <x:v>Link aus expliziter Data-Availability-Statement</x:v>
+        <x:v>Link aus expliziter Data-Availability-Statement; 6 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
@@ -5343,7 +5359,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ48" s="31" t="str">
-        <x:v>Titel-/Autor:innen-Match (1.00)</x:v>
+        <x:v>Titel-/Autor:innen-Match (1.00); 9 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="34" customHeight="1">
@@ -7936,7 +7952,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ78" s="31" t="str">
-        <x:v>Link aus expliziter Data-Availability-Statement</x:v>
+        <x:v>Link aus expliziter Data-Availability-Statement; 6 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="34" customHeight="1">
@@ -10099,7 +10115,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ103" s="31" t="str">
-        <x:v>Link aus Data-Availability-Abschnitt des öffentlichen PuRe-Volltexts</x:v>
+        <x:v>Link aus Data-Availability-Abschnitt des öffentlichen PuRe-Volltexts; 1 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="34" customHeight="1">
@@ -11758,7 +11774,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ122" s="31" t="str">
-        <x:v>Link aus expliziter Data-Availability-Statement</x:v>
+        <x:v>Link aus expliziter Data-Availability-Statement; 6 Datendatei(en) über OSF-API bestätigt; Link aus expliziter Data-Availability-Statement</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="34" customHeight="1">
@@ -12130,19 +12146,27 @@
       <x:c r="J127" s="31" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="K127" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K127" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L127" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M127" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N127" s="37" t="str"/>
-      <x:c r="O127" s="31" t="str"/>
-      <x:c r="P127" s="31" t="str"/>
-      <x:c r="Q127" s="31" t="str"/>
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="N127" s="37" t="str">
+        <x:v>https://github.com/predictive-clinical-neuroscience/PCNtoolkit-demo/tree/main/tutorials/Long_NM</x:v>
+      </x:c>
+      <x:c r="O127" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P127" s="31" t="str">
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="Q127" s="31" t="str">
+        <x:v>HTTP 200; HTTP</x:v>
+      </x:c>
       <x:c r="R127" s="37" t="str"/>
       <x:c r="S127" s="31" t="str"/>
       <x:c r="T127" s="31" t="str"/>
@@ -12179,10 +12203,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY127" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ127" s="31" t="str">
-        <x:v>Verlagsseite nennt keine eindeutige vorhandene Datenausgabe</x:v>
+        <x:v>Strukturierte eLife-Data-Availability-Aussage mit öffentlichem Datensatzlink; 32 Datendatei(en) über GitHub-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="34" customHeight="1">
@@ -12896,19 +12920,27 @@
       <x:c r="J136" s="31" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="K136" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K136" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L136" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M136" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N136" s="37" t="str"/>
-      <x:c r="O136" s="31" t="str"/>
-      <x:c r="P136" s="31" t="str"/>
-      <x:c r="Q136" s="31" t="str"/>
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="N136" s="37" t="str">
+        <x:v>https://services.informs.org/dataset/mnsc/download.php?doi=mnsc.2022.03362</x:v>
+      </x:c>
+      <x:c r="O136" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P136" s="39" t="str">
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="Q136" s="31" t="str">
+        <x:v>HTTP 200; Playwright</x:v>
+      </x:c>
       <x:c r="R136" s="37" t="str"/>
       <x:c r="S136" s="31" t="str"/>
       <x:c r="T136" s="31" t="str"/>
@@ -12945,10 +12977,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY136" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>Playwright</x:v>
       </x:c>
       <x:c r="AZ136" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Offizielles INFORMS-Replikationsarchiv mit geprüften Datendateien</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="34" customHeight="1">
@@ -14006,19 +14038,27 @@
       <x:c r="J149" s="31" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="K149" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K149" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L149" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M149" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N149" s="37" t="str"/>
-      <x:c r="O149" s="31" t="str"/>
-      <x:c r="P149" s="31" t="str"/>
-      <x:c r="Q149" s="31" t="str"/>
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="N149" s="37" t="str">
+        <x:v>https://services.informs.org/dataset/mnsc/download.php?doi=mnsc.2022.00652</x:v>
+      </x:c>
+      <x:c r="O149" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P149" s="39" t="str">
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="Q149" s="31" t="str">
+        <x:v>HTTP 200; Playwright</x:v>
+      </x:c>
       <x:c r="R149" s="37" t="str"/>
       <x:c r="S149" s="31" t="str"/>
       <x:c r="T149" s="31" t="str"/>
@@ -14055,10 +14095,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY149" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>Playwright</x:v>
       </x:c>
       <x:c r="AZ149" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Offizielles INFORMS-Replikationsarchiv mit geprüften Datendateien</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="34" customHeight="1">
@@ -16212,7 +16252,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ174" s="31" t="str">
-        <x:v>Identischer normalisierter Titel und starke Autor:innenüberschneidung mit item_3686548; Titel-/Autor:innen-Match (1.00)</x:v>
+        <x:v>Identischer normalisierter Titel und starke Autor:innenüberschneidung mit item_3686548; Titel-/Autor:innen-Match (1.00); 208 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="34" customHeight="1">
@@ -16306,7 +16346,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ175" s="31" t="str">
-        <x:v>Link aus expliziter Data-Availability-Statement</x:v>
+        <x:v>Link aus expliziter Data-Availability-Statement; 1 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="34" customHeight="1">
@@ -19686,7 +19726,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ214" s="31" t="str">
-        <x:v>Identischer normalisierter Titel und starke Autor:innenüberschneidung mit item_3657005; Link aus expliziter Data-Availability-Statement</x:v>
+        <x:v>Identischer normalisierter Titel und starke Autor:innenüberschneidung mit item_3657005; Link aus expliziter Data-Availability-Statement; 6 Datendatei(en) über OSF-API bestätigt; Identischer normalisierter Titel und starke Autor:innenüberschneidung mit item_3657005; Link aus expliziter Data-Availability-Statement</x:v>
       </x:c>
     </x:row>
     <x:row r="215" ht="34" customHeight="1">
@@ -20408,19 +20448,27 @@
       <x:c r="J223" s="31" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="K223" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K223" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L223" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M223" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N223" s="37" t="str"/>
-      <x:c r="O223" s="31" t="str"/>
-      <x:c r="P223" s="31" t="str"/>
-      <x:c r="Q223" s="31" t="str"/>
+        <x:v>offen über View-only-Link</x:v>
+      </x:c>
+      <x:c r="N223" s="37" t="str">
+        <x:v>https://osf.io/z34es/?view_only=634f9aba0001450d8baef233da73a1a4</x:v>
+      </x:c>
+      <x:c r="O223" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P223" s="39" t="str">
+        <x:v>offen über View-only-Link</x:v>
+      </x:c>
+      <x:c r="Q223" s="31" t="str">
+        <x:v>HTTP 200; HTTP</x:v>
+      </x:c>
       <x:c r="R223" s="37" t="str"/>
       <x:c r="S223" s="31" t="str"/>
       <x:c r="T223" s="31" t="str"/>
@@ -20457,10 +20505,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY223" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ223" s="31" t="str">
-        <x:v>Dataset-Treffer ohne hinreichend engen Publikationsbezug (0.09)</x:v>
+        <x:v>Wiley-Datenverfügbarkeitsaussage mit rekursiv geprüften OSF-Datendateien; 2 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="224" ht="34" customHeight="1">
@@ -20892,7 +20940,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ228" s="31" t="str">
-        <x:v>Link aus expliziter Data-Availability-Statement</x:v>
+        <x:v>Link aus expliziter Data-Availability-Statement; 3 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="229" ht="34" customHeight="1">
@@ -21012,19 +21060,27 @@
       <x:c r="J230" s="31" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="K230" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K230" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L230" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M230" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N230" s="37" t="str"/>
-      <x:c r="O230" s="31" t="str"/>
-      <x:c r="P230" s="31" t="str"/>
-      <x:c r="Q230" s="31" t="str"/>
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="N230" s="37" t="str">
+        <x:v>https://services.informs.org/dataset/mnsc/download.php?doi=mnsc.2023.4838</x:v>
+      </x:c>
+      <x:c r="O230" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P230" s="39" t="str">
+        <x:v>Zustimmung/E-Mail erforderlich</x:v>
+      </x:c>
+      <x:c r="Q230" s="31" t="str">
+        <x:v>HTTP 200; Playwright</x:v>
+      </x:c>
       <x:c r="R230" s="37" t="str"/>
       <x:c r="S230" s="31" t="str"/>
       <x:c r="T230" s="31" t="str"/>
@@ -21061,10 +21117,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY230" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>Playwright</x:v>
       </x:c>
       <x:c r="AZ230" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Offizielles INFORMS-Replikationsarchiv mit geprüften Datendateien</x:v>
       </x:c>
     </x:row>
     <x:row r="231" ht="34" customHeight="1">
@@ -21610,19 +21666,27 @@
       <x:c r="J237" s="31" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="K237" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K237" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L237" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M237" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N237" s="37" t="str"/>
-      <x:c r="O237" s="31" t="str"/>
-      <x:c r="P237" s="31" t="str"/>
-      <x:c r="Q237" s="31" t="str"/>
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="N237" s="37" t="str">
+        <x:v>https://osf.io/rgeq8</x:v>
+      </x:c>
+      <x:c r="O237" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P237" s="31" t="str">
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="Q237" s="31" t="str">
+        <x:v>HTTP 200; HTTP</x:v>
+      </x:c>
       <x:c r="R237" s="37" t="str"/>
       <x:c r="S237" s="31" t="str"/>
       <x:c r="T237" s="31" t="str"/>
@@ -21659,10 +21723,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY237" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ237" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Bereits auditierter Datensatz einer stark identifizierten Publikationsfassung; 3 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="238" ht="34" customHeight="1">
@@ -22944,7 +23008,7 @@
         <x:v>HTTP</x:v>
       </x:c>
       <x:c r="AZ252" s="31" t="str">
-        <x:v>Link aus Data-Availability-Abschnitt des öffentlichen PuRe-Volltexts</x:v>
+        <x:v>Link aus Data-Availability-Abschnitt des öffentlichen PuRe-Volltexts; 3 Datendatei(en) über OSF-API bestätigt</x:v>
       </x:c>
     </x:row>
     <x:row r="253" ht="34" customHeight="1">
@@ -23756,19 +23820,27 @@
       <x:c r="J262" s="31" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="K262" s="33" t="str">
-        <x:v>nein</x:v>
+      <x:c r="K262" s="32" t="str">
+        <x:v>ja</x:v>
       </x:c>
       <x:c r="L262" s="41" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M262" s="31" t="str">
-        <x:v>kein verifizierter Datenlink</x:v>
-      </x:c>
-      <x:c r="N262" s="37" t="str"/>
-      <x:c r="O262" s="31" t="str"/>
-      <x:c r="P262" s="31" t="str"/>
-      <x:c r="Q262" s="31" t="str"/>
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="N262" s="37" t="str">
+        <x:v>https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/SPJFJ5</x:v>
+      </x:c>
+      <x:c r="O262" s="31" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="P262" s="31" t="str">
+        <x:v>offen</x:v>
+      </x:c>
+      <x:c r="Q262" s="31" t="str">
+        <x:v>HTTP 202; Playwright</x:v>
+      </x:c>
       <x:c r="R262" s="37" t="str"/>
       <x:c r="S262" s="31" t="str"/>
       <x:c r="T262" s="31" t="str"/>
@@ -23805,10 +23877,10 @@
         <x:v>2026-07-15</x:v>
       </x:c>
       <x:c r="AY262" s="31" t="str">
-        <x:v>HTTP + Playwright-Audit</x:v>
+        <x:v>Playwright</x:v>
       </x:c>
       <x:c r="AZ262" s="31" t="str">
-        <x:v>Keine verifizierten Forschungsdaten gefunden</x:v>
+        <x:v>Bereits auditierter Datensatz einer stark identifizierten Publikationsfassung</x:v>
       </x:c>
     </x:row>
     <x:row r="263" ht="34" customHeight="1">
@@ -25360,7 +25432,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a17a9d77f2d4de0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14488b790c734584"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25420,13 +25492,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="29" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D4" s="29" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D4" s="29" t="n">
-        <x:v>5</x:v>
-      </x:c>
       <x:c r="E4" s="48" t="n">
-        <x:v>0.4444444444444444</x:v>
+        <x:v>0.5555555555555556</x:v>
       </x:c>
       <x:c r="F4" s="29" t="n">
         <x:v>3</x:v>
@@ -25443,13 +25515,13 @@
         <x:v>118</x:v>
       </x:c>
       <x:c r="C5" s="31" t="n">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="31" t="n">
-        <x:v>99</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E5" s="49" t="n">
-        <x:v>0.16101694915254236</x:v>
+        <x:v>0.1864406779661017</x:v>
       </x:c>
       <x:c r="F5" s="31" t="n">
         <x:v>11</x:v>
@@ -25558,19 +25630,19 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="C10" s="31" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D10" s="31" t="n">
-        <x:v>43</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E10" s="49" t="n">
-        <x:v>0.0851063829787234</x:v>
+        <x:v>0.14893617021276595</x:v>
       </x:c>
       <x:c r="F10" s="31" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G10" s="31" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
@@ -25604,19 +25676,19 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="C12" s="31" t="n">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D12" s="31" t="n">
-        <x:v>59</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E12" s="49" t="n">
-        <x:v>0.20270270270270271</x:v>
+        <x:v>0.22972972972972974</x:v>
       </x:c>
       <x:c r="F12" s="31" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="G12" s="31" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
@@ -25675,7 +25747,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff384e42b90b4a7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbef09546561d4f55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>